<commit_message>
chore: namuna shablon yangilandi (manzilli-template.xlsx)
</commit_message>
<xml_diff>
--- a/assets/templates/manzilli-template.xlsx
+++ b/assets/templates/manzilli-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SH\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F73D9F6F-FD18-4770-9E74-3B6349666D9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45220B7E-9BF0-47DC-88C1-10FFD0A18408}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -828,11 +828,11 @@
       <c r="E6" s="17"/>
       <c r="F6" s="17"/>
       <c r="G6" s="17"/>
-      <c r="H6" s="17"/>
-      <c r="I6" s="14">
-        <f>SUM(I7:I173)</f>
+      <c r="H6" s="14">
+        <f>SUM(H7:H173)</f>
         <v>0</v>
       </c>
+      <c r="I6" s="14"/>
       <c r="J6" s="15" t="s">
         <v>14</v>
       </c>

</xml_diff>

<commit_message>
chore: namuna shablon yangilandi (v3)
</commit_message>
<xml_diff>
--- a/assets/templates/manzilli-template.xlsx
+++ b/assets/templates/manzilli-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SH\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45220B7E-9BF0-47DC-88C1-10FFD0A18408}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F68E6973-0B0E-4BED-86F0-58E0D08D0066}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -725,9 +725,16 @@
   <cols>
     <col min="1" max="1" width="5.85546875" customWidth="1"/>
     <col min="2" max="2" width="14.5703125" hidden="1" customWidth="1"/>
-    <col min="3" max="3" width="20.5703125" customWidth="1"/>
-    <col min="4" max="4" width="16" style="1" customWidth="1"/>
-    <col min="5" max="12" width="28.5703125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="43.140625" customWidth="1"/>
+    <col min="4" max="4" width="34" style="1" customWidth="1"/>
+    <col min="5" max="5" width="33.7109375" style="1" customWidth="1"/>
+    <col min="6" max="6" width="30.42578125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="29.85546875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="32.7109375" style="1" customWidth="1"/>
+    <col min="9" max="9" width="28.5703125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="45.28515625" style="1" customWidth="1"/>
+    <col min="11" max="11" width="31.42578125" style="1" customWidth="1"/>
+    <col min="12" max="12" width="32.28515625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
@@ -839,7 +846,7 @@
       <c r="K6" s="17"/>
       <c r="L6" s="17"/>
     </row>
-    <row r="7" spans="1:12" ht="65.099999999999994" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" ht="75.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>1</v>
       </c>
@@ -857,7 +864,7 @@
       <c r="K7" s="7"/>
       <c r="L7" s="7"/>
     </row>
-    <row r="8" spans="1:12" ht="65.099999999999994" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" ht="75.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>2</v>
       </c>
@@ -875,7 +882,7 @@
       <c r="K8" s="7"/>
       <c r="L8" s="7"/>
     </row>
-    <row r="9" spans="1:12" ht="65.099999999999994" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" ht="75.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>3</v>
       </c>
@@ -893,7 +900,7 @@
       <c r="K9" s="7"/>
       <c r="L9" s="7"/>
     </row>
-    <row r="10" spans="1:12" ht="65.099999999999994" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" ht="75.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>4</v>
       </c>
@@ -911,7 +918,7 @@
       <c r="K10" s="7"/>
       <c r="L10" s="7"/>
     </row>
-    <row r="11" spans="1:12" ht="65.099999999999994" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" ht="75.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>5</v>
       </c>
@@ -929,7 +936,7 @@
       <c r="K11" s="7"/>
       <c r="L11" s="7"/>
     </row>
-    <row r="12" spans="1:12" ht="65.099999999999994" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" ht="75.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>6</v>
       </c>
@@ -947,7 +954,7 @@
       <c r="K12" s="7"/>
       <c r="L12" s="7"/>
     </row>
-    <row r="13" spans="1:12" ht="65.099999999999994" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" ht="75.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>7</v>
       </c>
@@ -965,7 +972,7 @@
       <c r="K13" s="7"/>
       <c r="L13" s="7"/>
     </row>
-    <row r="14" spans="1:12" ht="65.099999999999994" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12" ht="75.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>8</v>
       </c>
@@ -1000,7 +1007,7 @@
     <mergeCell ref="C4:C5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="31" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="25" orientation="portrait" r:id="rId1"/>
   <ignoredErrors>
     <ignoredError sqref="A4:B4 A5:B5 A1:B1 C5 C1:C3 A3:B3 B2 A7:B14 B6" numberStoredAsText="1"/>
   </ignoredErrors>

</xml_diff>